<commit_message>
Procurement re-issued: OSB fixed with 3.1x50 coil nails (P-11a), not staples
</commit_message>
<xml_diff>
--- a/docs/procurement/P3-PR-01 Procurement Schedule C01.xlsx
+++ b/docs/procurement/P3-PR-01 Procurement Schedule C01.xlsx
@@ -973,7 +973,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>50mm staples (box of 5,000)</t>
+          <t>3.1x50mm coil nails (box of 2,500)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -982,11 +982,11 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>GF panels: 0.65; FF panels: 0.54; Gable panels: 0.25</t>
+          <t>GF panels: 1.3; FF panels: 1.09; Gable panels: 0.5</t>
         </is>
       </c>
     </row>
@@ -3404,7 +3404,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>50mm staples (box of 5,000)</t>
+          <t>3.1x50mm coil nails (box of 2,500)</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -3421,11 +3421,11 @@
         <v>2952</v>
       </c>
       <c r="F67" t="n">
-        <v>0.65</v>
+        <v>1.3</v>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>2952 staples (@150 edges / 300 field) +10%</t>
+          <t>2952 OSB coil nails (@150 edges / 300 field) +10%</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
@@ -3443,7 +3443,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>50mm staples (box of 5,000)</t>
+          <t>3.1x50mm coil nails (box of 2,500)</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -3460,11 +3460,11 @@
         <v>2474</v>
       </c>
       <c r="F68" t="n">
-        <v>0.54</v>
+        <v>1.09</v>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>2474 staples (@150 edges / 300 field) +10%</t>
+          <t>2474 OSB coil nails (@150 edges / 300 field) +10%</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -3482,7 +3482,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>50mm staples (box of 5,000)</t>
+          <t>3.1x50mm coil nails (box of 2,500)</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -3499,11 +3499,11 @@
         <v>1127</v>
       </c>
       <c r="F69" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>1127 staples (@150 edges / 300 field) +10%</t>
+          <t>1127 OSB coil nails (@150 edges / 300 field) +10%</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
@@ -3517,7 +3517,7 @@
       <c r="A70" s="3" t="inlineStr"/>
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>TOTAL 50mm staples (box of 5,000)</t>
+          <t>TOTAL 3.1x50mm coil nails (box of 2,500)</t>
         </is>
       </c>
       <c r="C70" s="3" t="inlineStr">
@@ -3528,7 +3528,7 @@
       <c r="D70" s="3" t="inlineStr"/>
       <c r="E70" s="3" t="inlineStr"/>
       <c r="F70" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G70" s="3" t="inlineStr"/>
       <c r="H70" s="3" t="inlineStr"/>
@@ -4049,7 +4049,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Nails 3 x 90 ring-shank per joint / noggin end, multi-ply @150 staggered (both sides &gt; 2 ply, 3 lots &gt; 3 ply), boxes 2,500. Staples 50mm @150 edges / 300 field, boxes 5,000. No VCL, no mineral wool. PIR 120 to external walls only.</t>
+          <t>Nails 3 x 90 ring-shank per joint / noggin end, multi-ply @150 staggered (both sides &gt; 2 ply, 3 lots &gt; 3 ply), boxes 2,500. OSB: 3.1x50 coil nails @150 edges / 300 field, boxes 2,500 (P-11a). No VCL, no mineral wool. PIR 120 to external walls only.</t>
         </is>
       </c>
     </row>

</xml_diff>